<commit_message>
records-templates: update export workbooks
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/records/dataExchange_groups.xlsx
+++ b/owlcms/src/main/resources/templates/records/dataExchange_groups.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms_v23\owlcms\src\main\resources\templates\records\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms4\owlcms\src\main\resources\templates\records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D89E9C-54AA-4A5B-B9B4-B8F05CF2B340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FA42CD5-322F-4B23-9B6C-9D4FADECB7EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3900" yWindow="3900" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Records" sheetId="1" r:id="rId1"/>
@@ -62,83 +62,6 @@
         </r>
       </text>
     </comment>
-    <comment ref="H2" authorId="0" shapeId="0" xr:uid="{C6FF4C17-205A-4117-9526-D4356C492D3F}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>owlcms:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-for non-heavyweight category use a number
-45 59 55 64 ...
-for heavyweight category use 999</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K2" authorId="0" shapeId="0" xr:uid="{E929A3F5-8334-4A41-8BFE-3F8D0356CC97}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>owlcms:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Columns from K to O are optional and are not used by the system
-You can leave them empty.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P2" authorId="0" shapeId="0" xr:uid="{17BBEB5E-9C88-41B3-B3AF-34E640F0734C}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">owlcms:
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Column P indicates the session in which the record was set.
-This indicates a new record established in the current competition.</t>
-        </r>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
@@ -233,9 +156,6 @@
     <t>${r.groupNameString}</t>
   </si>
   <si>
-    <t>${r.bwCatString}</t>
-  </si>
-  <si>
     <t>M/F</t>
   </si>
   <si>
@@ -246,13 +166,16 @@
   </si>
   <si>
     <t>${r.event}</t>
+  </si>
+  <si>
+    <t>${r.bwCatUpper}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -271,19 +194,6 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
@@ -385,6 +295,122 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>7937</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>158750</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="8109656" cy="609013"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CBF6D8FE-B103-D844-2545-C5CAA2602421}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4135437" y="857250"/>
+          <a:ext cx="8109656" cy="609013"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFF00"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>Column I</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> : </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>For non-heavyweight category use a number</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>60, 65, 70, 75, 85, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>...</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>for heavyweight category use 999</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>Columns from K to O are optional and are not used by the system You can leave them empty.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>Column P indicates the session in which the record was set. This indicates a new provisional  record established in the current competition.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -717,7 +743,7 @@
         <v>9</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E1" s="13" t="s">
         <v>10</v>
@@ -756,7 +782,7 @@
         <v>13</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
@@ -782,7 +808,7 @@
         <v>19</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="I2" s="7" t="s">
         <v>20</v>
@@ -803,13 +829,13 @@
         <v>27</v>
       </c>
       <c r="O2" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="P2" s="7" t="s">
         <v>28</v>
       </c>
       <c r="Q2" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -1228,7 +1254,7 @@
       <c r="O29" s="7"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="2">
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1:G1048576" xr:uid="{53FB7450-D8BD-4FB4-A0E8-29CC05EF8875}">
       <formula1>0</formula1>
       <formula2>250</formula2>
@@ -1237,13 +1263,10 @@
       <formula1>0</formula1>
       <formula2>120</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H1:H1048576" xr:uid="{905FFAC0-C9A6-475E-9DE4-6B5BF21663BF}">
-      <formula1>0</formula1>
-      <formula2>999</formula2>
-    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>